<commit_message>
Soluciona IndexError en exportacion Excel e introduce sample_data realista
</commit_message>
<xml_diff>
--- a/sample_data/Control_sample.xlsx
+++ b/sample_data/Control_sample.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -463,13 +463,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6.977202529401594</v>
+        <v>10.01</v>
       </c>
       <c r="D2" t="n">
-        <v>9.877252526587355</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>101</v>
       </c>
       <c r="F2" t="n">
         <v>1</v>
@@ -486,20 +486,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EEA1</t>
+          <t>Cav1</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>16.73459925230384</v>
+        <v>10.02</v>
       </c>
       <c r="D3" t="n">
-        <v>22.11448847993024</v>
+        <v>10</v>
       </c>
       <c r="E3" t="n">
+        <v>101</v>
+      </c>
+      <c r="F3" t="n">
         <v>2</v>
-      </c>
-      <c r="F3" t="n">
-        <v>1</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -517,16 +517,16 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18.3835517762038</v>
+        <v>10.03</v>
       </c>
       <c r="D4" t="n">
-        <v>13.1088998659516</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
+        <v>101</v>
+      </c>
+      <c r="F4" t="n">
         <v>3</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -540,20 +540,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>EEA1</t>
+          <t>Cav1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>16.79255546477007</v>
+        <v>10.04</v>
       </c>
       <c r="D5" t="n">
-        <v>6.889341773787754</v>
+        <v>10</v>
       </c>
       <c r="E5" t="n">
+        <v>101</v>
+      </c>
+      <c r="F5" t="n">
         <v>4</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -571,16 +571,16 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>9.643848225781248</v>
+        <v>10.05</v>
       </c>
       <c r="D6" t="n">
-        <v>6.950205968045021</v>
+        <v>10</v>
       </c>
       <c r="E6" t="n">
+        <v>101</v>
+      </c>
+      <c r="F6" t="n">
         <v>5</v>
-      </c>
-      <c r="F6" t="n">
-        <v>3</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -594,20 +594,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EEA1</t>
+          <t>Cav1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>18.87840540171376</v>
+        <v>10.06</v>
       </c>
       <c r="D7" t="n">
-        <v>8.699696201410237</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
+        <v>101</v>
+      </c>
+      <c r="F7" t="n">
         <v>6</v>
-      </c>
-      <c r="F7" t="n">
-        <v>3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -625,16 +625,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>20.10420266460993</v>
+        <v>10.07</v>
       </c>
       <c r="D8" t="n">
-        <v>18.34564315885984</v>
+        <v>10</v>
       </c>
       <c r="E8" t="n">
+        <v>101</v>
+      </c>
+      <c r="F8" t="n">
         <v>7</v>
-      </c>
-      <c r="F8" t="n">
-        <v>4</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -648,20 +648,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EEA1</t>
+          <t>Cav1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>17.82657772374314</v>
+        <v>10.08</v>
       </c>
       <c r="D9" t="n">
-        <v>6.970075195933168</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
+        <v>101</v>
+      </c>
+      <c r="F9" t="n">
         <v>8</v>
-      </c>
-      <c r="F9" t="n">
-        <v>4</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -679,16 +679,16 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9.290296115524646</v>
+        <v>10.09</v>
       </c>
       <c r="D10" t="n">
-        <v>14.21279566296058</v>
+        <v>10</v>
       </c>
       <c r="E10" t="n">
+        <v>101</v>
+      </c>
+      <c r="F10" t="n">
         <v>9</v>
-      </c>
-      <c r="F10" t="n">
-        <v>5</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -706,16 +706,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>15.09695092970877</v>
+        <v>10.06</v>
       </c>
       <c r="D11" t="n">
-        <v>23.1823500500672</v>
+        <v>10.02</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>201</v>
       </c>
       <c r="F11" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -725,24 +725,24 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>EEA1</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10.07</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="E12" t="n">
+        <v>201</v>
+      </c>
+      <c r="F12" t="n">
         <v>2</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Cav1</t>
-        </is>
-      </c>
-      <c r="C12" t="n">
-        <v>23.30520850664459</v>
-      </c>
-      <c r="D12" t="n">
-        <v>7.095307943757582</v>
-      </c>
-      <c r="E12" t="n">
-        <v>11</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -760,16 +760,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>8.359807783116377</v>
+        <v>10.08</v>
       </c>
       <c r="D13" t="n">
-        <v>19.89737657875201</v>
+        <v>10.02</v>
       </c>
       <c r="E13" t="n">
-        <v>12</v>
+        <v>201</v>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -779,24 +779,24 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cav1</t>
+          <t>EEA1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>19.3076924668956</v>
+        <v>10.09</v>
       </c>
       <c r="D14" t="n">
-        <v>21.60646101416402</v>
+        <v>10.02</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>201</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -814,16 +814,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>16.20831275519275</v>
+        <v>10.1</v>
       </c>
       <c r="D15" t="n">
-        <v>6.603550047302223</v>
+        <v>10.02</v>
       </c>
       <c r="E15" t="n">
-        <v>14</v>
+        <v>201</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -833,24 +833,24 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cav1</t>
+          <t>EEA1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>8.690958805696383</v>
+        <v>10.11</v>
       </c>
       <c r="D16" t="n">
-        <v>12.92851695411105</v>
+        <v>10.02</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>201</v>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -868,16 +868,16 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>9.922813145980241</v>
+        <v>10.12</v>
       </c>
       <c r="D17" t="n">
-        <v>7.846779594050847</v>
+        <v>10.02</v>
       </c>
       <c r="E17" t="n">
-        <v>16</v>
+        <v>201</v>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -887,24 +887,24 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cav1</t>
+          <t>EEA1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>16.29737014989955</v>
+        <v>10.13</v>
       </c>
       <c r="D18" t="n">
-        <v>23.0801190953582</v>
+        <v>10.02</v>
       </c>
       <c r="E18" t="n">
-        <v>17</v>
+        <v>201</v>
       </c>
       <c r="F18" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -922,72 +922,18 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20.51533909481632</v>
+        <v>10.14</v>
       </c>
       <c r="D19" t="n">
-        <v>13.08803892407852</v>
+        <v>10.02</v>
       </c>
       <c r="E19" t="n">
-        <v>18</v>
+        <v>201</v>
       </c>
       <c r="F19" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G19" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Cav1</t>
-        </is>
-      </c>
-      <c r="C20" t="n">
-        <v>19.16974692525865</v>
-      </c>
-      <c r="D20" t="n">
-        <v>9.67092475726947</v>
-      </c>
-      <c r="E20" t="n">
-        <v>19</v>
-      </c>
-      <c r="F20" t="n">
-        <v>5</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Control</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>EEA1</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>18.5428150477294</v>
-      </c>
-      <c r="D21" t="n">
-        <v>23.59568325327163</v>
-      </c>
-      <c r="E21" t="n">
-        <v>20</v>
-      </c>
-      <c r="F21" t="n">
-        <v>5</v>
-      </c>
-      <c r="G21" t="inlineStr">
         <is>
           <t>Control</t>
         </is>

</xml_diff>